<commit_message>
Add Names and Adjust the Template
</commit_message>
<xml_diff>
--- a/MacroDashboard Versions/Economic Dashboard V1-Template.xlsx
+++ b/MacroDashboard Versions/Economic Dashboard V1-Template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Desktop\Duke Research Opportunity\Prof. Aguilar Macro Dashboard\MacroDashBoard\MacroDashboard Versions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{366CBBCB-2A06-406B-8618-B1D967D335F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E926AF1-FA10-4E7E-99C3-6EC144CA259E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -359,9 +359,6 @@
     <t>Macro Dashboard</t>
   </si>
   <si>
-    <t>Mike Aguilar | mike.aguilar@duke.edu | www.market-observatory.com</t>
-  </si>
-  <si>
     <t>Source: All data collected via FRED from the St. Louis Fed</t>
   </si>
   <si>
@@ -552,6 +549,11 @@
   </si>
   <si>
     <t>TWEXBGSMTH</t>
+  </si>
+  <si>
+    <t>Mike Aguilar | mike.aguilar@duke.edu |
+Jacky Yang    | jacky.yang@duke.edu    |
+www.market-observatory.com</t>
   </si>
 </sst>
 </file>
@@ -717,7 +719,7 @@
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -848,6 +850,15 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1148,7 +1159,7 @@
   <sheetPr codeName="Sheet1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U80"/>
+  <dimension ref="A1:U55"/>
   <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="15.75" x14ac:dyDescent="0.5"/>
   <cols>
     <col min="1" max="1" width="29.3984375" style="30" customWidth="1"/>
@@ -1203,7 +1214,7 @@
         <v>80</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D2" s="10" t="s">
         <v>25</v>
@@ -1234,7 +1245,7 @@
         <v>80</v>
       </c>
       <c r="N2" s="18" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="O2" s="10" t="s">
         <v>25</v>
@@ -1263,7 +1274,7 @@
         <v>12</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="6" t="s">
@@ -1292,7 +1303,7 @@
         <v>41</v>
       </c>
       <c r="M3" s="15" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="N3" s="7"/>
       <c r="O3" s="6" t="s">
@@ -1320,7 +1331,7 @@
     <row r="4" spans="1:21" x14ac:dyDescent="0.5">
       <c r="A4" s="34"/>
       <c r="B4" s="15" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C4" s="7"/>
       <c r="D4" s="6" t="s">
@@ -1347,7 +1358,7 @@
       <c r="K4" s="5"/>
       <c r="L4" s="28"/>
       <c r="M4" s="15" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="N4" s="7"/>
       <c r="O4" s="6" t="s">
@@ -1377,7 +1388,7 @@
         <v>13</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C5" s="7"/>
       <c r="D5" s="6" t="s">
@@ -1406,7 +1417,7 @@
         <v>50</v>
       </c>
       <c r="M5" s="15" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="N5" s="7"/>
       <c r="O5" s="6" t="s">
@@ -1434,7 +1445,7 @@
     <row r="6" spans="1:21" x14ac:dyDescent="0.5">
       <c r="A6" s="33"/>
       <c r="B6" s="15" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="6" t="s">
@@ -1463,7 +1474,7 @@
         <v>8</v>
       </c>
       <c r="M6" s="15" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="N6" s="7"/>
       <c r="O6" s="6" t="s">
@@ -1493,7 +1504,7 @@
         <v>81</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="6" t="s">
@@ -1522,7 +1533,7 @@
         <v>86</v>
       </c>
       <c r="M7" s="15" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="N7" s="7"/>
       <c r="O7" s="6" t="s">
@@ -1561,27 +1572,27 @@
       <c r="E8" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="F8" s="24">
-        <v>1</v>
-      </c>
-      <c r="G8" s="24">
-        <v>1</v>
-      </c>
-      <c r="H8" s="24">
-        <v>1</v>
-      </c>
-      <c r="I8" s="24">
-        <v>1</v>
-      </c>
-      <c r="J8" s="24">
-        <v>1</v>
-      </c>
-      <c r="K8" s="5"/>
+      <c r="F8" s="6">
+        <v>1</v>
+      </c>
+      <c r="G8" s="6">
+        <v>1</v>
+      </c>
+      <c r="H8" s="6">
+        <v>1</v>
+      </c>
+      <c r="I8" s="6">
+        <v>1</v>
+      </c>
+      <c r="J8" s="45">
+        <v>1</v>
+      </c>
+      <c r="K8" s="46"/>
       <c r="L8" s="28" t="s">
         <v>40</v>
       </c>
       <c r="M8" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="N8" s="7"/>
       <c r="O8" s="6" t="s">
@@ -1611,7 +1622,7 @@
         <v>32</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C9" s="7"/>
       <c r="D9" s="6" t="s">
@@ -1640,7 +1651,7 @@
         <v>45</v>
       </c>
       <c r="M9" s="15" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="N9" s="7"/>
       <c r="O9" s="6" t="s">
@@ -1668,7 +1679,7 @@
     <row r="10" spans="1:21" x14ac:dyDescent="0.5">
       <c r="A10" s="33"/>
       <c r="B10" s="15" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C10" s="7"/>
       <c r="D10" s="6" t="s">
@@ -1697,7 +1708,7 @@
         <v>47</v>
       </c>
       <c r="M10" s="15" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="N10" s="7"/>
       <c r="O10" s="6" t="s">
@@ -1727,7 +1738,7 @@
         <v>28</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C11" s="7"/>
       <c r="D11" s="6" t="s">
@@ -1756,7 +1767,7 @@
         <v>46</v>
       </c>
       <c r="M11" s="15" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="N11" s="7"/>
       <c r="O11" s="6" t="s">
@@ -1784,7 +1795,7 @@
     <row r="12" spans="1:21" x14ac:dyDescent="0.5">
       <c r="A12" s="33"/>
       <c r="B12" s="15" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C12" s="7"/>
       <c r="D12" s="6" t="s">
@@ -1813,7 +1824,7 @@
         <v>82</v>
       </c>
       <c r="M12" s="15" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="N12" s="7"/>
       <c r="O12" s="6" t="s">
@@ -1843,7 +1854,7 @@
         <v>29</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C13" s="7"/>
       <c r="D13" s="6" t="s">
@@ -1872,7 +1883,7 @@
         <v>42</v>
       </c>
       <c r="M13" s="15" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="N13" s="7"/>
       <c r="O13" s="6" t="s">
@@ -1900,7 +1911,7 @@
     <row r="14" spans="1:21" x14ac:dyDescent="0.5">
       <c r="A14" s="34"/>
       <c r="B14" s="15" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C14" s="7"/>
       <c r="D14" s="6" t="s">
@@ -1929,7 +1940,7 @@
         <v>48</v>
       </c>
       <c r="M14" s="15" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="N14" s="7"/>
       <c r="O14" s="6" t="s">
@@ -1959,7 +1970,7 @@
         <v>30</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C15" s="7"/>
       <c r="D15" s="6" t="s">
@@ -1988,7 +1999,7 @@
         <v>84</v>
       </c>
       <c r="M15" s="15" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="N15" s="7"/>
       <c r="O15" s="6" t="s">
@@ -2016,7 +2027,7 @@
     <row r="16" spans="1:21" x14ac:dyDescent="0.5">
       <c r="A16" s="33"/>
       <c r="B16" s="15" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C16" s="7"/>
       <c r="D16" s="6" t="s">
@@ -2057,7 +2068,7 @@
         <v>53</v>
       </c>
       <c r="B17" s="15" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C17" s="7"/>
       <c r="D17" s="6" t="s">
@@ -2116,7 +2127,7 @@
     <row r="18" spans="1:21" x14ac:dyDescent="0.5">
       <c r="A18" s="33"/>
       <c r="B18" s="15" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C18" s="7"/>
       <c r="D18" s="6" t="s">
@@ -2145,7 +2156,7 @@
         <v>22</v>
       </c>
       <c r="M18" s="15" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="N18" s="7"/>
       <c r="O18" s="6" t="s">
@@ -2175,7 +2186,7 @@
         <v>61</v>
       </c>
       <c r="B19" s="15" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C19" s="7"/>
       <c r="D19" s="6" t="s">
@@ -2202,7 +2213,7 @@
       <c r="K19" s="5"/>
       <c r="L19" s="28"/>
       <c r="M19" s="15" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="N19" s="7"/>
       <c r="O19" s="6" t="s">
@@ -2230,7 +2241,7 @@
     <row r="20" spans="1:21" x14ac:dyDescent="0.5">
       <c r="A20" s="33"/>
       <c r="B20" s="15" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C20" s="7"/>
       <c r="D20" s="6" t="s">
@@ -2259,7 +2270,7 @@
         <v>23</v>
       </c>
       <c r="M20" s="15" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="N20" s="7"/>
       <c r="O20" s="6" t="s">
@@ -2289,7 +2300,7 @@
         <v>62</v>
       </c>
       <c r="B21" s="15" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C21" s="7"/>
       <c r="D21" s="6" t="s">
@@ -2316,7 +2327,7 @@
       <c r="K21" s="5"/>
       <c r="L21" s="28"/>
       <c r="M21" s="15" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="N21" s="7"/>
       <c r="O21" s="6" t="s">
@@ -2375,7 +2386,7 @@
         <v>38</v>
       </c>
       <c r="M22" s="15" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="N22" s="7"/>
       <c r="O22" s="6" t="s">
@@ -2429,7 +2440,7 @@
       </c>
       <c r="K23" s="5"/>
       <c r="M23" s="15" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="N23" s="7"/>
       <c r="O23" s="6" t="s">
@@ -2459,7 +2470,7 @@
         <v>94</v>
       </c>
       <c r="B24" s="15" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C24" s="7"/>
       <c r="D24" s="6" t="s">
@@ -2488,7 +2499,7 @@
         <v>57</v>
       </c>
       <c r="M24" s="15" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="N24" s="7"/>
       <c r="O24" s="6" t="s">
@@ -2518,7 +2529,7 @@
         <v>95</v>
       </c>
       <c r="B25" s="15" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C25" s="7"/>
       <c r="D25" s="6" t="s">
@@ -2545,7 +2556,7 @@
       <c r="K25" s="5"/>
       <c r="L25" s="28"/>
       <c r="M25" s="15" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="N25" s="7"/>
       <c r="O25" s="6" t="s">
@@ -2575,7 +2586,7 @@
         <v>96</v>
       </c>
       <c r="B26" s="15" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C26" s="7"/>
       <c r="D26" s="6" t="s">
@@ -2604,7 +2615,7 @@
         <v>58</v>
       </c>
       <c r="M26" s="15" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="N26" s="7"/>
       <c r="O26" s="6" t="s">
@@ -2634,7 +2645,7 @@
         <v>97</v>
       </c>
       <c r="B27" s="15" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C27" s="7"/>
       <c r="D27" s="6" t="s">
@@ -2661,7 +2672,7 @@
       <c r="K27" s="5"/>
       <c r="L27" s="28"/>
       <c r="M27" s="15" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="N27" s="7"/>
       <c r="O27" s="6" t="s">
@@ -2691,7 +2702,7 @@
         <v>14</v>
       </c>
       <c r="B28" s="15" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C28" s="7"/>
       <c r="D28" s="6" t="s">
@@ -2720,7 +2731,7 @@
         <v>59</v>
       </c>
       <c r="M28" s="15" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="N28" s="7"/>
       <c r="O28" s="6" t="s">
@@ -2748,7 +2759,7 @@
     <row r="29" spans="1:21" x14ac:dyDescent="0.5">
       <c r="A29" s="33"/>
       <c r="B29" s="15" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C29" s="7"/>
       <c r="D29" s="6" t="s">
@@ -2777,7 +2788,7 @@
         <v>78</v>
       </c>
       <c r="M29" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="N29" s="7"/>
       <c r="O29" s="6" t="s">
@@ -2807,7 +2818,7 @@
         <v>68</v>
       </c>
       <c r="B30" s="15" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C30" s="7"/>
       <c r="D30" s="6" t="s">
@@ -2836,7 +2847,7 @@
         <v>79</v>
       </c>
       <c r="M30" s="15" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="N30" s="7"/>
       <c r="O30" s="6" t="s">
@@ -2864,7 +2875,7 @@
     <row r="31" spans="1:21" x14ac:dyDescent="0.5">
       <c r="A31" s="33"/>
       <c r="B31" s="15" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C31" s="7"/>
       <c r="D31" s="6" t="s">
@@ -2893,7 +2904,7 @@
         <v>72</v>
       </c>
       <c r="M31" s="7" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="N31" s="7"/>
       <c r="O31" s="6" t="s">
@@ -2923,7 +2934,7 @@
         <v>10</v>
       </c>
       <c r="B32" s="15" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C32" s="7"/>
       <c r="D32" s="6" t="s">
@@ -2950,7 +2961,7 @@
       <c r="K32" s="5"/>
       <c r="L32" s="28"/>
       <c r="M32" s="7" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="N32" s="7"/>
       <c r="O32" s="6" t="s">
@@ -2978,7 +2989,7 @@
     <row r="33" spans="1:21" ht="31.5" x14ac:dyDescent="0.5">
       <c r="A33" s="33"/>
       <c r="B33" s="15" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C33" s="7"/>
       <c r="D33" s="6" t="s">
@@ -3007,7 +3018,7 @@
         <v>74</v>
       </c>
       <c r="M33" s="15" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="N33" s="7"/>
       <c r="O33" s="6" t="s">
@@ -3037,7 +3048,7 @@
         <v>69</v>
       </c>
       <c r="B34" s="15" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C34" s="7"/>
       <c r="D34" s="6" t="s">
@@ -3064,7 +3075,7 @@
       <c r="K34" s="5"/>
       <c r="L34" s="28"/>
       <c r="M34" s="15" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="N34" s="7"/>
       <c r="O34" s="6" t="s">
@@ -3094,7 +3105,7 @@
         <v>83</v>
       </c>
       <c r="B35" s="15" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C35" s="7"/>
       <c r="D35" s="6" t="s">
@@ -3120,10 +3131,10 @@
       </c>
       <c r="K35" s="5"/>
       <c r="L35" s="28" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="M35" s="15" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="N35" s="7"/>
       <c r="O35" s="6" t="s">
@@ -3153,7 +3164,7 @@
         <v>15</v>
       </c>
       <c r="B36" s="15" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C36" s="7"/>
       <c r="D36" s="6" t="s">
@@ -3180,7 +3191,7 @@
       <c r="K36" s="5"/>
       <c r="L36" s="28"/>
       <c r="M36" s="15" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="N36" s="7"/>
       <c r="O36" s="6" t="s">
@@ -3208,7 +3219,7 @@
     <row r="37" spans="1:21" x14ac:dyDescent="0.5">
       <c r="A37" s="33"/>
       <c r="B37" s="15" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C37" s="7"/>
       <c r="D37" s="6" t="s">
@@ -3237,7 +3248,7 @@
         <v>75</v>
       </c>
       <c r="M37" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="N37" s="7"/>
       <c r="O37" s="6" t="s">
@@ -3267,7 +3278,7 @@
         <v>64</v>
       </c>
       <c r="B38" s="15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C38" s="7"/>
       <c r="D38" s="6" t="s">
@@ -3294,7 +3305,7 @@
       <c r="K38" s="5"/>
       <c r="L38" s="28"/>
       <c r="M38" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="N38" s="7"/>
       <c r="O38" s="6" t="s">
@@ -3322,7 +3333,7 @@
     <row r="39" spans="1:21" ht="31.5" x14ac:dyDescent="0.5">
       <c r="A39" s="33"/>
       <c r="B39" s="15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C39" s="7"/>
       <c r="D39" s="6" t="s">
@@ -3351,7 +3362,7 @@
         <v>76</v>
       </c>
       <c r="M39" s="15" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="N39" s="7"/>
       <c r="O39" s="6" t="s">
@@ -3381,7 +3392,7 @@
         <v>66</v>
       </c>
       <c r="B40" s="15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C40" s="7"/>
       <c r="D40" s="6" t="s">
@@ -3408,7 +3419,7 @@
       <c r="K40" s="5"/>
       <c r="L40" s="28"/>
       <c r="M40" s="15" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="N40" s="7"/>
       <c r="O40" s="6" t="s">
@@ -3436,7 +3447,7 @@
     <row r="41" spans="1:21" x14ac:dyDescent="0.5">
       <c r="A41" s="33"/>
       <c r="B41" s="15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C41" s="7"/>
       <c r="D41" s="6" t="s">
@@ -3465,7 +3476,7 @@
         <v>54</v>
       </c>
       <c r="M41" s="15" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="N41" s="7"/>
       <c r="O41" s="6" t="s">
@@ -3495,7 +3506,7 @@
         <v>67</v>
       </c>
       <c r="B42" s="15" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C42" s="7"/>
       <c r="D42" s="6" t="s">
@@ -3522,7 +3533,7 @@
       <c r="K42" s="7"/>
       <c r="L42" s="28"/>
       <c r="M42" s="15" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="N42" s="7"/>
       <c r="O42" s="6" t="s">
@@ -3550,7 +3561,7 @@
     <row r="43" spans="1:21" x14ac:dyDescent="0.5">
       <c r="A43" s="33"/>
       <c r="B43" s="15" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C43" s="7"/>
       <c r="D43" s="6" t="s">
@@ -3579,7 +3590,7 @@
         <v>55</v>
       </c>
       <c r="M43" s="15" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="N43" s="7"/>
       <c r="O43" s="6" t="s">
@@ -3609,7 +3620,7 @@
         <v>16</v>
       </c>
       <c r="B44" s="15" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C44" s="7"/>
       <c r="D44" s="6" t="s">
@@ -3636,7 +3647,7 @@
       <c r="K44" s="5"/>
       <c r="L44" s="28"/>
       <c r="M44" s="15" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="N44" s="7"/>
       <c r="O44" s="6" t="s">
@@ -3664,7 +3675,7 @@
     <row r="45" spans="1:21" x14ac:dyDescent="0.5">
       <c r="A45" s="33"/>
       <c r="B45" s="15" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C45" s="7"/>
       <c r="D45" s="6" t="s">
@@ -3705,7 +3716,7 @@
         <v>33</v>
       </c>
       <c r="B46" s="15" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C46" s="7"/>
       <c r="D46" s="6" t="s">
@@ -3764,7 +3775,7 @@
     <row r="47" spans="1:21" x14ac:dyDescent="0.5">
       <c r="A47" s="33"/>
       <c r="B47" s="15" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C47" s="7"/>
       <c r="D47" s="6" t="s">
@@ -3793,7 +3804,7 @@
         <v>18</v>
       </c>
       <c r="M47" s="15" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="N47" s="7"/>
       <c r="O47" s="6" t="s">
@@ -3823,7 +3834,7 @@
         <v>34</v>
       </c>
       <c r="B48" s="15" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C48" s="7"/>
       <c r="D48" s="6" t="s">
@@ -3852,7 +3863,7 @@
         <v>17</v>
       </c>
       <c r="M48" s="15" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="N48" s="7"/>
       <c r="O48" s="6" t="s">
@@ -3880,7 +3891,7 @@
     <row r="49" spans="1:21" x14ac:dyDescent="0.5">
       <c r="A49" s="33"/>
       <c r="B49" s="15" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C49" s="7"/>
       <c r="D49" s="6" t="s">
@@ -3909,7 +3920,7 @@
         <v>19</v>
       </c>
       <c r="M49" s="15" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="N49" s="7"/>
       <c r="O49" s="6" t="s">
@@ -3939,7 +3950,7 @@
         <v>52</v>
       </c>
       <c r="B50" s="15" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C50" s="7"/>
       <c r="D50" s="6" t="s">
@@ -3968,7 +3979,7 @@
         <v>20</v>
       </c>
       <c r="M50" s="15" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="N50" s="7"/>
       <c r="O50" s="6" t="s">
@@ -3996,7 +4007,7 @@
     <row r="51" spans="1:21" ht="31.5" x14ac:dyDescent="0.5">
       <c r="A51" s="33"/>
       <c r="B51" s="15" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C51" s="7"/>
       <c r="D51" s="6" t="s">
@@ -4025,7 +4036,7 @@
         <v>21</v>
       </c>
       <c r="M51" s="15" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="N51" s="7"/>
       <c r="O51" s="6" t="s">
@@ -4066,7 +4077,7 @@
         <v>60</v>
       </c>
       <c r="M52" s="17" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="N52" s="20"/>
       <c r="O52" s="9" t="s">
@@ -4096,7 +4107,7 @@
         <v>70</v>
       </c>
       <c r="B53" s="40" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C53" s="7"/>
       <c r="D53" s="6"/>
@@ -4120,7 +4131,7 @@
     </row>
     <row r="54" spans="1:21" ht="21" x14ac:dyDescent="0.5">
       <c r="A54" s="37" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B54" s="15"/>
       <c r="C54" s="7"/>
@@ -4143,9 +4154,9 @@
       <c r="T54" s="6"/>
       <c r="U54" s="6"/>
     </row>
-    <row r="55" spans="1:21" ht="21" x14ac:dyDescent="0.5">
-      <c r="A55" s="37" t="s">
-        <v>100</v>
+    <row r="55" spans="1:21" ht="31.5" x14ac:dyDescent="0.5">
+      <c r="A55" s="47" t="s">
+        <v>164</v>
       </c>
       <c r="B55" s="15"/>
       <c r="C55" s="7"/>
@@ -4168,9 +4179,6 @@
       <c r="T55" s="6"/>
       <c r="U55" s="6"/>
     </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.5">
-      <c r="A80" s="4"/>
-    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:U1"/>

</xml_diff>